<commit_message>
feat: refine SAV conversion workflow
</commit_message>
<xml_diff>
--- a/docs/sav_mapping_template.xlsx
+++ b/docs/sav_mapping_template.xlsx
@@ -77,7 +77,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve">字段</t>
+          <t xml:space="preserve">原则</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -89,130 +89,179 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t xml:space="preserve">source_col</t>
+          <t xml:space="preserve">自动命名</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t xml:space="preserve">原始 Excel 列号</t>
+          <t xml:space="preserve">默认按 question_id / 列角色推断，例如 q13、q23_text、q20_01</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t xml:space="preserve">source_header</t>
+          <t xml:space="preserve">自动类型</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t xml:space="preserve">原始列头</t>
+          <t xml:space="preserve">默认根据列值和映射关系推断 numeric/string，可人工调整</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t xml:space="preserve">question_id</t>
+          <t xml:space="preserve">自动保留</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t xml:space="preserve">问卷题号，如 Q20</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">spss_name</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">建议的 SAV 变量名，可人工调整</t>
-        </is>
-      </c>
-    </row>
+          <t xml:space="preserve">除 flow 变量外默认 keep=1，可人工修改</t>
+        </is>
+      </c>
+    </row>
+    <row r="11"/>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t xml:space="preserve">variable_label</t>
+          <t xml:space="preserve">字段</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t xml:space="preserve">建议的 SAV 变量标签</t>
+          <t xml:space="preserve">说明</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">var_type</t>
+          <t xml:space="preserve">source_col</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t xml:space="preserve">numeric/string</t>
+          <t xml:space="preserve">原始 Excel 列号</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t xml:space="preserve">measure</t>
+          <t xml:space="preserve">source_header</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t xml:space="preserve">nominal/ordinal/scale</t>
+          <t xml:space="preserve">原始列头</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t xml:space="preserve">role</t>
+          <t xml:space="preserve">question_id</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t xml:space="preserve">single/multi_binary/open_text/meta 等</t>
+          <t xml:space="preserve">问卷题号，如 Q20</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t xml:space="preserve">keep</t>
+          <t xml:space="preserve">spss_name</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t xml:space="preserve">1=输出到最终 SAV；0=默认不输出</t>
+          <t xml:space="preserve">建议的 SAV 变量名，可人工调整</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t xml:space="preserve">transform_rule</t>
+          <t xml:space="preserve">variable_label</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t xml:space="preserve">脚本执行字段转换时使用的规则标记</t>
+          <t xml:space="preserve">建议的 SAV 变量标签</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
+          <t xml:space="preserve">var_type</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">numeric/string</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">measure</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">nominal/ordinal/scale</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">role</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">single/multi_binary/open_text/meta 等</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">keep</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1=输出到最终 SAV；0=默认不输出</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">transform_rule</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">脚本执行字段转换时使用的规则标记</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
           <t xml:space="preserve">notes</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="B23" t="inlineStr">
         <is>
           <t xml:space="preserve">补充说明</t>
         </is>
@@ -320,7 +369,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t xml:space="preserve">meta_submit_id</t>
+          <t xml:space="preserve">meta_a</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -377,7 +426,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t xml:space="preserve">meta_status</t>
+          <t xml:space="preserve">meta_b</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -402,7 +451,7 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t xml:space="preserve">0</t>
+          <t xml:space="preserve">1</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -903,7 +952,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t xml:space="preserve">q03_terminate_flag</t>
+          <t xml:space="preserve">q3_flow</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1367,7 +1416,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t xml:space="preserve">q05_terminate_flag</t>
+          <t xml:space="preserve">q5_flow</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1429,7 +1478,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t xml:space="preserve">q06_gender</t>
+          <t xml:space="preserve">q6</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1486,7 +1535,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t xml:space="preserve">q07_age_band</t>
+          <t xml:space="preserve">q7</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1501,7 +1550,7 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t xml:space="preserve">ordinal</t>
+          <t xml:space="preserve">nominal</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
@@ -1543,7 +1592,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t xml:space="preserve">q08_terminate_flag</t>
+          <t xml:space="preserve">q8_flow</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1940,7 +1989,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t xml:space="preserve">q10_terminate_flag</t>
+          <t xml:space="preserve">q10_flow</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -2203,7 +2252,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t xml:space="preserve">q12_terminate_flag</t>
+          <t xml:space="preserve">q12_flow</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -2265,7 +2314,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t xml:space="preserve">q13_brand_main</t>
+          <t xml:space="preserve">q13</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -2322,7 +2371,7 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t xml:space="preserve">q15_drink_frequency</t>
+          <t xml:space="preserve">q15</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -2337,7 +2386,7 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t xml:space="preserve">ordinal</t>
+          <t xml:space="preserve">nominal</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
@@ -3126,7 +3175,7 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q16-9.您通常在什么场景下喝啤酒？【多选题】_其他是否填写</t>
+          <t xml:space="preserve">Q16-9.您通常在什么场景下喝啤酒？【多选题】_其他，请注明_是否填写</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
@@ -3193,7 +3242,7 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q16-9.您通常在什么场景下喝啤酒？【多选题】_其他文本</t>
+          <t xml:space="preserve">Q16-9.您通常在什么场景下喝啤酒？【多选题】_其他，请注明_填写文本</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
@@ -3250,7 +3299,7 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t xml:space="preserve">q17_price_band</t>
+          <t xml:space="preserve">q17</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -3265,7 +3314,7 @@
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t xml:space="preserve">ordinal</t>
+          <t xml:space="preserve">nominal</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
@@ -3307,7 +3356,7 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t xml:space="preserve">q18_taste_preference</t>
+          <t xml:space="preserve">q18</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -3364,7 +3413,7 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t xml:space="preserve">q19_attention_text</t>
+          <t xml:space="preserve">q19_text</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -4302,7 +4351,7 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q20-13.在选购啤酒时，除了品牌和价格之外，您最关注以下哪些因素？【多选题，限选5项】_其他是否填写</t>
+          <t xml:space="preserve">Q20-13.在选购啤酒时，除了品牌和价格之外，您最关注以下哪些因素？【多选题，限选5项】_其他，请注明_是否填写</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
@@ -4369,7 +4418,7 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q20-13.在选购啤酒时，除了品牌和价格之外，您最关注以下哪些因素？【多选题，限选5项】_其他文本</t>
+          <t xml:space="preserve">Q20-13.在选购啤酒时，除了品牌和价格之外，您最关注以下哪些因素？【多选题，限选5项】_其他，请注明_填写文本</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
@@ -4426,7 +4475,7 @@
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t xml:space="preserve">q22_like_level</t>
+          <t xml:space="preserve">q22</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
@@ -4441,7 +4490,7 @@
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t xml:space="preserve">ordinal</t>
+          <t xml:space="preserve">nominal</t>
         </is>
       </c>
       <c r="J65" t="inlineStr">
@@ -4483,7 +4532,7 @@
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t xml:space="preserve">q23_like_reason_text</t>
+          <t xml:space="preserve">q23_text</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
@@ -4540,7 +4589,7 @@
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t xml:space="preserve">q24_dislike_reason_text</t>
+          <t xml:space="preserve">q24_text</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
@@ -4597,7 +4646,7 @@
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t xml:space="preserve">q25_uniqueness</t>
+          <t xml:space="preserve">q25</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
@@ -4612,7 +4661,7 @@
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t xml:space="preserve">ordinal</t>
+          <t xml:space="preserve">nominal</t>
         </is>
       </c>
       <c r="J68" t="inlineStr">
@@ -4654,7 +4703,7 @@
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t xml:space="preserve">q26_purchase_intent</t>
+          <t xml:space="preserve">q26</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
@@ -4669,7 +4718,7 @@
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t xml:space="preserve">ordinal</t>
+          <t xml:space="preserve">nominal</t>
         </is>
       </c>
       <c r="J69" t="inlineStr">
@@ -4711,7 +4760,7 @@
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t xml:space="preserve">q27a_price_too_low</t>
+          <t xml:space="preserve">q27_text</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
@@ -4721,17 +4770,17 @@
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t xml:space="preserve">numeric</t>
+          <t xml:space="preserve">string</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t xml:space="preserve">scale</t>
+          <t xml:space="preserve">nominal</t>
         </is>
       </c>
       <c r="J70" t="inlineStr">
         <is>
-          <t xml:space="preserve">open_numeric</t>
+          <t xml:space="preserve">open_text</t>
         </is>
       </c>
       <c r="K70" t="inlineStr">
@@ -4768,7 +4817,7 @@
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t xml:space="preserve">q27b_price_bargain</t>
+          <t xml:space="preserve">q27_text_2</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
@@ -4778,17 +4827,17 @@
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t xml:space="preserve">numeric</t>
+          <t xml:space="preserve">string</t>
         </is>
       </c>
       <c r="I71" t="inlineStr">
         <is>
-          <t xml:space="preserve">scale</t>
+          <t xml:space="preserve">nominal</t>
         </is>
       </c>
       <c r="J71" t="inlineStr">
         <is>
-          <t xml:space="preserve">open_numeric</t>
+          <t xml:space="preserve">open_text</t>
         </is>
       </c>
       <c r="K71" t="inlineStr">
@@ -4825,7 +4874,7 @@
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t xml:space="preserve">q27c_price_high_ok</t>
+          <t xml:space="preserve">q27_text_3</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
@@ -4835,17 +4884,17 @@
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t xml:space="preserve">numeric</t>
+          <t xml:space="preserve">string</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
         <is>
-          <t xml:space="preserve">scale</t>
+          <t xml:space="preserve">nominal</t>
         </is>
       </c>
       <c r="J72" t="inlineStr">
         <is>
-          <t xml:space="preserve">open_numeric</t>
+          <t xml:space="preserve">open_text</t>
         </is>
       </c>
       <c r="K72" t="inlineStr">
@@ -4882,7 +4931,7 @@
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t xml:space="preserve">q27d_price_too_high</t>
+          <t xml:space="preserve">q27_text_4</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
@@ -4892,17 +4941,17 @@
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t xml:space="preserve">numeric</t>
+          <t xml:space="preserve">string</t>
         </is>
       </c>
       <c r="I73" t="inlineStr">
         <is>
-          <t xml:space="preserve">scale</t>
+          <t xml:space="preserve">nominal</t>
         </is>
       </c>
       <c r="J73" t="inlineStr">
         <is>
-          <t xml:space="preserve">open_numeric</t>
+          <t xml:space="preserve">open_text</t>
         </is>
       </c>
       <c r="K73" t="inlineStr">
@@ -4939,7 +4988,7 @@
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t xml:space="preserve">q28_preferred_beer</t>
+          <t xml:space="preserve">q28</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
@@ -4996,7 +5045,7 @@
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t xml:space="preserve">q29_preferred_beer_reason_text</t>
+          <t xml:space="preserve">q29_text</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
@@ -5053,7 +5102,7 @@
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t xml:space="preserve">q31_preferred_opening</t>
+          <t xml:space="preserve">q31</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
@@ -5110,7 +5159,7 @@
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t xml:space="preserve">q32_preferred_opening_reason_text</t>
+          <t xml:space="preserve">q32_text</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
@@ -5167,7 +5216,7 @@
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t xml:space="preserve">q34_occupation</t>
+          <t xml:space="preserve">q34</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
@@ -5224,7 +5273,7 @@
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t xml:space="preserve">q35_education</t>
+          <t xml:space="preserve">q35</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
@@ -5239,7 +5288,7 @@
       </c>
       <c r="I79" t="inlineStr">
         <is>
-          <t xml:space="preserve">ordinal</t>
+          <t xml:space="preserve">nominal</t>
         </is>
       </c>
       <c r="J79" t="inlineStr">
@@ -5281,7 +5330,7 @@
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t xml:space="preserve">q36_household_income</t>
+          <t xml:space="preserve">q36</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
@@ -5296,7 +5345,7 @@
       </c>
       <c r="I80" t="inlineStr">
         <is>
-          <t xml:space="preserve">ordinal</t>
+          <t xml:space="preserve">nominal</t>
         </is>
       </c>
       <c r="J80" t="inlineStr">
@@ -5338,7 +5387,7 @@
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t xml:space="preserve">q37_living_status</t>
+          <t xml:space="preserve">q37</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
@@ -6611,7 +6660,7 @@
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q38- | 28.以下娱乐爱好，请选择与您符合的：【多选题】 |_其他是否填写</t>
+          <t xml:space="preserve">Q38- | 28.以下娱乐爱好，请选择与您符合的：【多选题】 | _其他，请注明_是否填写</t>
         </is>
       </c>
       <c r="H100" t="inlineStr">
@@ -6678,7 +6727,7 @@
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q38- | 28.以下娱乐爱好，请选择与您符合的：【多选题】 |_其他文本</t>
+          <t xml:space="preserve">Q38- | 28.以下娱乐爱好，请选择与您符合的：【多选题】 | _其他，请注明_填写文本</t>
         </is>
       </c>
       <c r="H101" t="inlineStr">
@@ -6735,7 +6784,7 @@
       </c>
       <c r="F102" t="inlineStr">
         <is>
-          <t xml:space="preserve">q39_end_flag</t>
+          <t xml:space="preserve">q39</t>
         </is>
       </c>
       <c r="G102" t="inlineStr">
@@ -6792,7 +6841,7 @@
       </c>
       <c r="F103" t="inlineStr">
         <is>
-          <t xml:space="preserve">meta_extended_field</t>
+          <t xml:space="preserve">meta_cu</t>
         </is>
       </c>
       <c r="G103" t="inlineStr">
@@ -6817,7 +6866,7 @@
       </c>
       <c r="K103" t="inlineStr">
         <is>
-          <t xml:space="preserve">0</t>
+          <t xml:space="preserve">1</t>
         </is>
       </c>
       <c r="M103" t="inlineStr">
@@ -6849,7 +6898,7 @@
       </c>
       <c r="F104" t="inlineStr">
         <is>
-          <t xml:space="preserve">meta_user_id</t>
+          <t xml:space="preserve">meta_cv</t>
         </is>
       </c>
       <c r="G104" t="inlineStr">
@@ -6859,7 +6908,7 @@
       </c>
       <c r="H104" t="inlineStr">
         <is>
-          <t xml:space="preserve">numeric</t>
+          <t xml:space="preserve">string</t>
         </is>
       </c>
       <c r="I104" t="inlineStr">
@@ -6906,7 +6955,7 @@
       </c>
       <c r="F105" t="inlineStr">
         <is>
-          <t xml:space="preserve">meta_update_user</t>
+          <t xml:space="preserve">meta_cw</t>
         </is>
       </c>
       <c r="G105" t="inlineStr">
@@ -6931,7 +6980,7 @@
       </c>
       <c r="K105" t="inlineStr">
         <is>
-          <t xml:space="preserve">0</t>
+          <t xml:space="preserve">1</t>
         </is>
       </c>
       <c r="M105" t="inlineStr">
@@ -6963,7 +7012,7 @@
       </c>
       <c r="F106" t="inlineStr">
         <is>
-          <t xml:space="preserve">meta_submit_time</t>
+          <t xml:space="preserve">meta_cx</t>
         </is>
       </c>
       <c r="G106" t="inlineStr">
@@ -7020,7 +7069,7 @@
       </c>
       <c r="F107" t="inlineStr">
         <is>
-          <t xml:space="preserve">meta_update_time</t>
+          <t xml:space="preserve">meta_cy</t>
         </is>
       </c>
       <c r="G107" t="inlineStr">
@@ -7077,7 +7126,7 @@
       </c>
       <c r="F108" t="inlineStr">
         <is>
-          <t xml:space="preserve">meta_audio_url</t>
+          <t xml:space="preserve">meta_cz</t>
         </is>
       </c>
       <c r="G108" t="inlineStr">
@@ -7102,7 +7151,7 @@
       </c>
       <c r="K108" t="inlineStr">
         <is>
-          <t xml:space="preserve">0</t>
+          <t xml:space="preserve">1</t>
         </is>
       </c>
       <c r="M108" t="inlineStr">
@@ -7134,7 +7183,7 @@
       </c>
       <c r="F109" t="inlineStr">
         <is>
-          <t xml:space="preserve">meta_duration</t>
+          <t xml:space="preserve">meta_da</t>
         </is>
       </c>
       <c r="G109" t="inlineStr">
@@ -7191,7 +7240,7 @@
       </c>
       <c r="F110" t="inlineStr">
         <is>
-          <t xml:space="preserve">meta_start_time</t>
+          <t xml:space="preserve">meta_db</t>
         </is>
       </c>
       <c r="G110" t="inlineStr">
@@ -7248,7 +7297,7 @@
       </c>
       <c r="F111" t="inlineStr">
         <is>
-          <t xml:space="preserve">meta_pending_task_id</t>
+          <t xml:space="preserve">meta_dc</t>
         </is>
       </c>
       <c r="G111" t="inlineStr">
@@ -7273,7 +7322,7 @@
       </c>
       <c r="K111" t="inlineStr">
         <is>
-          <t xml:space="preserve">0</t>
+          <t xml:space="preserve">1</t>
         </is>
       </c>
       <c r="M111" t="inlineStr">
@@ -7305,7 +7354,7 @@
       </c>
       <c r="F112" t="inlineStr">
         <is>
-          <t xml:space="preserve">meta_last_review_task_id</t>
+          <t xml:space="preserve">meta_dd</t>
         </is>
       </c>
       <c r="G112" t="inlineStr">
@@ -7330,7 +7379,7 @@
       </c>
       <c r="K112" t="inlineStr">
         <is>
-          <t xml:space="preserve">0</t>
+          <t xml:space="preserve">1</t>
         </is>
       </c>
       <c r="M112" t="inlineStr">
@@ -7362,7 +7411,7 @@
       </c>
       <c r="F113" t="inlineStr">
         <is>
-          <t xml:space="preserve">meta_hierarchy_path</t>
+          <t xml:space="preserve">meta_de</t>
         </is>
       </c>
       <c r="G113" t="inlineStr">
@@ -7387,7 +7436,7 @@
       </c>
       <c r="K113" t="inlineStr">
         <is>
-          <t xml:space="preserve">0</t>
+          <t xml:space="preserve">1</t>
         </is>
       </c>
       <c r="M113" t="inlineStr">
@@ -7419,7 +7468,7 @@
       </c>
       <c r="F114" t="inlineStr">
         <is>
-          <t xml:space="preserve">meta_pending_user</t>
+          <t xml:space="preserve">meta_df</t>
         </is>
       </c>
       <c r="G114" t="inlineStr">
@@ -7444,7 +7493,7 @@
       </c>
       <c r="K114" t="inlineStr">
         <is>
-          <t xml:space="preserve">0</t>
+          <t xml:space="preserve">1</t>
         </is>
       </c>
       <c r="M114" t="inlineStr">
@@ -7476,7 +7525,7 @@
       </c>
       <c r="F115" t="inlineStr">
         <is>
-          <t xml:space="preserve">meta_address</t>
+          <t xml:space="preserve">meta_dg</t>
         </is>
       </c>
       <c r="G115" t="inlineStr">
@@ -7533,7 +7582,7 @@
       </c>
       <c r="F116" t="inlineStr">
         <is>
-          <t xml:space="preserve">meta_username</t>
+          <t xml:space="preserve">meta_dh</t>
         </is>
       </c>
       <c r="G116" t="inlineStr">
@@ -7982,7 +8031,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t xml:space="preserve">q03_terminate_flag</t>
+          <t xml:space="preserve">q3_flow</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -8333,7 +8382,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t xml:space="preserve">q05_terminate_flag</t>
+          <t xml:space="preserve">q5_flow</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -8360,7 +8409,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t xml:space="preserve">q06_gender</t>
+          <t xml:space="preserve">q6</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -8387,7 +8436,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t xml:space="preserve">q06_gender</t>
+          <t xml:space="preserve">q6</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -8414,7 +8463,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t xml:space="preserve">q07_age_band</t>
+          <t xml:space="preserve">q7</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -8441,7 +8490,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t xml:space="preserve">q07_age_band</t>
+          <t xml:space="preserve">q7</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -8468,7 +8517,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t xml:space="preserve">q07_age_band</t>
+          <t xml:space="preserve">q7</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -8495,7 +8544,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t xml:space="preserve">q07_age_band</t>
+          <t xml:space="preserve">q7</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -8522,7 +8571,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t xml:space="preserve">q07_age_band</t>
+          <t xml:space="preserve">q7</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -8549,7 +8598,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t xml:space="preserve">q08_terminate_flag</t>
+          <t xml:space="preserve">q8_flow</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -8846,7 +8895,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t xml:space="preserve">q10_terminate_flag</t>
+          <t xml:space="preserve">q10_flow</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -9035,7 +9084,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t xml:space="preserve">q12_terminate_flag</t>
+          <t xml:space="preserve">q12_flow</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -9062,7 +9111,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t xml:space="preserve">q13_brand_main</t>
+          <t xml:space="preserve">q13</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -9089,7 +9138,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t xml:space="preserve">q13_brand_main</t>
+          <t xml:space="preserve">q13</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -9116,7 +9165,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t xml:space="preserve">q13_brand_main</t>
+          <t xml:space="preserve">q13</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -9143,7 +9192,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t xml:space="preserve">q15_drink_frequency</t>
+          <t xml:space="preserve">q15</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -9170,7 +9219,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t xml:space="preserve">q15_drink_frequency</t>
+          <t xml:space="preserve">q15</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -9197,7 +9246,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t xml:space="preserve">q15_drink_frequency</t>
+          <t xml:space="preserve">q15</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -9224,7 +9273,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t xml:space="preserve">q15_drink_frequency</t>
+          <t xml:space="preserve">q15</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -9251,7 +9300,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t xml:space="preserve">q15_drink_frequency</t>
+          <t xml:space="preserve">q15</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -9926,7 +9975,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t xml:space="preserve">q17_price_band</t>
+          <t xml:space="preserve">q17</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -9953,7 +10002,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t xml:space="preserve">q17_price_band</t>
+          <t xml:space="preserve">q17</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -9980,7 +10029,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t xml:space="preserve">q17_price_band</t>
+          <t xml:space="preserve">q17</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -10007,7 +10056,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t xml:space="preserve">q17_price_band</t>
+          <t xml:space="preserve">q17</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -10034,7 +10083,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t xml:space="preserve">q17_price_band</t>
+          <t xml:space="preserve">q17</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -10061,7 +10110,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t xml:space="preserve">q18_taste_preference</t>
+          <t xml:space="preserve">q18</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -10088,7 +10137,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t xml:space="preserve">q18_taste_preference</t>
+          <t xml:space="preserve">q18</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -10115,7 +10164,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t xml:space="preserve">q18_taste_preference</t>
+          <t xml:space="preserve">q18</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -10142,7 +10191,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t xml:space="preserve">q18_taste_preference</t>
+          <t xml:space="preserve">q18</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -10169,7 +10218,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t xml:space="preserve">q18_taste_preference</t>
+          <t xml:space="preserve">q18</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -10952,7 +11001,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t xml:space="preserve">q22_like_level</t>
+          <t xml:space="preserve">q22</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -10979,7 +11028,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t xml:space="preserve">q22_like_level</t>
+          <t xml:space="preserve">q22</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
@@ -11006,7 +11055,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t xml:space="preserve">q22_like_level</t>
+          <t xml:space="preserve">q22</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -11033,7 +11082,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t xml:space="preserve">q25_uniqueness</t>
+          <t xml:space="preserve">q25</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -11060,7 +11109,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t xml:space="preserve">q25_uniqueness</t>
+          <t xml:space="preserve">q25</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
@@ -11087,7 +11136,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t xml:space="preserve">q25_uniqueness</t>
+          <t xml:space="preserve">q25</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -11114,7 +11163,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t xml:space="preserve">q25_uniqueness</t>
+          <t xml:space="preserve">q25</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -11141,7 +11190,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t xml:space="preserve">q25_uniqueness</t>
+          <t xml:space="preserve">q25</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -11168,7 +11217,7 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t xml:space="preserve">q26_purchase_intent</t>
+          <t xml:space="preserve">q26</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
@@ -11195,7 +11244,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t xml:space="preserve">q26_purchase_intent</t>
+          <t xml:space="preserve">q26</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
@@ -11222,7 +11271,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t xml:space="preserve">q26_purchase_intent</t>
+          <t xml:space="preserve">q26</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
@@ -11249,7 +11298,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t xml:space="preserve">q26_purchase_intent</t>
+          <t xml:space="preserve">q26</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -11276,7 +11325,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t xml:space="preserve">q28_preferred_beer</t>
+          <t xml:space="preserve">q28</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
@@ -11303,7 +11352,7 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t xml:space="preserve">q28_preferred_beer</t>
+          <t xml:space="preserve">q28</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
@@ -11330,7 +11379,7 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t xml:space="preserve">q31_preferred_opening</t>
+          <t xml:space="preserve">q31</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
@@ -11357,7 +11406,7 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t xml:space="preserve">q31_preferred_opening</t>
+          <t xml:space="preserve">q31</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
@@ -11384,7 +11433,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t xml:space="preserve">q34_occupation</t>
+          <t xml:space="preserve">q34</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
@@ -11411,7 +11460,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t xml:space="preserve">q34_occupation</t>
+          <t xml:space="preserve">q34</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -11438,7 +11487,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t xml:space="preserve">q34_occupation</t>
+          <t xml:space="preserve">q34</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
@@ -11465,7 +11514,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t xml:space="preserve">q34_occupation</t>
+          <t xml:space="preserve">q34</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
@@ -11492,7 +11541,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t xml:space="preserve">q34_occupation</t>
+          <t xml:space="preserve">q34</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
@@ -11519,7 +11568,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t xml:space="preserve">q34_occupation</t>
+          <t xml:space="preserve">q34</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
@@ -11546,7 +11595,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t xml:space="preserve">q34_occupation</t>
+          <t xml:space="preserve">q34</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
@@ -11573,7 +11622,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t xml:space="preserve">q34_occupation</t>
+          <t xml:space="preserve">q34</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
@@ -11600,7 +11649,7 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t xml:space="preserve">q34_occupation</t>
+          <t xml:space="preserve">q34</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
@@ -11627,7 +11676,7 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t xml:space="preserve">q34_occupation</t>
+          <t xml:space="preserve">q34</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
@@ -11654,7 +11703,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t xml:space="preserve">q34_occupation</t>
+          <t xml:space="preserve">q34</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
@@ -11681,7 +11730,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t xml:space="preserve">q34_occupation</t>
+          <t xml:space="preserve">q34</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
@@ -11708,7 +11757,7 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t xml:space="preserve">q34_occupation</t>
+          <t xml:space="preserve">q34</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
@@ -11735,7 +11784,7 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t xml:space="preserve">q34_occupation</t>
+          <t xml:space="preserve">q34</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
@@ -11762,7 +11811,7 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t xml:space="preserve">q34_occupation</t>
+          <t xml:space="preserve">q34</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
@@ -11789,7 +11838,7 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t xml:space="preserve">q34_occupation</t>
+          <t xml:space="preserve">q34</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
@@ -11816,7 +11865,7 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t xml:space="preserve">q34_occupation</t>
+          <t xml:space="preserve">q34</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
@@ -11843,7 +11892,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t xml:space="preserve">q34_occupation</t>
+          <t xml:space="preserve">q34</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
@@ -11870,7 +11919,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t xml:space="preserve">q34_occupation</t>
+          <t xml:space="preserve">q34</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
@@ -11897,7 +11946,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t xml:space="preserve">q34_occupation</t>
+          <t xml:space="preserve">q34</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
@@ -11924,7 +11973,7 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t xml:space="preserve">q34_occupation</t>
+          <t xml:space="preserve">q34</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
@@ -11951,7 +12000,7 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t xml:space="preserve">q34_occupation</t>
+          <t xml:space="preserve">q34</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
@@ -11978,7 +12027,7 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t xml:space="preserve">q34_occupation</t>
+          <t xml:space="preserve">q34</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
@@ -12005,7 +12054,7 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t xml:space="preserve">q35_education</t>
+          <t xml:space="preserve">q35</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
@@ -12032,7 +12081,7 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t xml:space="preserve">q35_education</t>
+          <t xml:space="preserve">q35</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
@@ -12059,7 +12108,7 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t xml:space="preserve">q35_education</t>
+          <t xml:space="preserve">q35</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
@@ -12086,7 +12135,7 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t xml:space="preserve">q35_education</t>
+          <t xml:space="preserve">q35</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
@@ -12113,7 +12162,7 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t xml:space="preserve">q35_education</t>
+          <t xml:space="preserve">q35</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
@@ -12140,7 +12189,7 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t xml:space="preserve">q35_education</t>
+          <t xml:space="preserve">q35</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
@@ -12167,7 +12216,7 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t xml:space="preserve">q36_household_income</t>
+          <t xml:space="preserve">q36</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
@@ -12194,7 +12243,7 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t xml:space="preserve">q36_household_income</t>
+          <t xml:space="preserve">q36</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
@@ -12221,7 +12270,7 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t xml:space="preserve">q36_household_income</t>
+          <t xml:space="preserve">q36</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
@@ -12248,7 +12297,7 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t xml:space="preserve">q36_household_income</t>
+          <t xml:space="preserve">q36</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
@@ -12275,7 +12324,7 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t xml:space="preserve">q36_household_income</t>
+          <t xml:space="preserve">q36</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
@@ -12302,7 +12351,7 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t xml:space="preserve">q36_household_income</t>
+          <t xml:space="preserve">q36</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
@@ -12329,7 +12378,7 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t xml:space="preserve">q36_household_income</t>
+          <t xml:space="preserve">q36</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
@@ -12356,7 +12405,7 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t xml:space="preserve">q36_household_income</t>
+          <t xml:space="preserve">q36</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
@@ -12383,7 +12432,7 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t xml:space="preserve">q36_household_income</t>
+          <t xml:space="preserve">q36</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
@@ -12410,7 +12459,7 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t xml:space="preserve">q36_household_income</t>
+          <t xml:space="preserve">q36</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
@@ -12437,7 +12486,7 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t xml:space="preserve">q36_household_income</t>
+          <t xml:space="preserve">q36</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
@@ -12464,7 +12513,7 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t xml:space="preserve">q37_living_status</t>
+          <t xml:space="preserve">q37</t>
         </is>
       </c>
       <c r="B182" t="inlineStr">
@@ -12491,7 +12540,7 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t xml:space="preserve">q37_living_status</t>
+          <t xml:space="preserve">q37</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
@@ -12518,7 +12567,7 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t xml:space="preserve">q37_living_status</t>
+          <t xml:space="preserve">q37</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
@@ -12545,7 +12594,7 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t xml:space="preserve">q37_living_status</t>
+          <t xml:space="preserve">q37</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
@@ -12572,7 +12621,7 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t xml:space="preserve">q37_living_status</t>
+          <t xml:space="preserve">q37</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
@@ -12599,7 +12648,7 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t xml:space="preserve">q37_living_status</t>
+          <t xml:space="preserve">q37</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
@@ -12626,7 +12675,7 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t xml:space="preserve">q37_living_status</t>
+          <t xml:space="preserve">q37</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
@@ -12653,7 +12702,7 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t xml:space="preserve">q37_living_status</t>
+          <t xml:space="preserve">q37</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
@@ -13706,7 +13755,7 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t xml:space="preserve">q39_end_flag</t>
+          <t xml:space="preserve">q39</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">

</xml_diff>